<commit_message>
Add category subtotals to cost estimate table
Each category now shows a subtotal row. Spreadsheet uses SUM formulas
per category; grand total sums the subtotal cells (no double-counting).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trip_costs.xlsx
+++ b/trip_costs.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,7 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font/>
     <font>
       <i val="1"/>
     </font>
@@ -44,7 +45,7 @@
       <color rgb="00888888"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +62,11 @@
         <fgColor rgb="00D5E8F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF3FB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -74,21 +80,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -454,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -489,235 +499,295 @@
       <c r="C2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>UA 108 IAD→MUC Jul 11 + OS135/UA53 VIE→IAD Jul 21 (4 people, Standard Economy)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>5422.52</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C4" s="8">
+        <f>SUM(C3:C3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Accommodation</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Munich — Holiday Inn Westpark, 2 nights (Jul 12–14)</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C6" s="5" t="n">
         <v>677.36</v>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+    <row r="7">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Königssee — Villa Alpenrausch, 3 nights (Jul 14–17) *</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
+    <row r="8">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Salzburg — Numa Vogelweider, 2 nights (Jul 17–19)</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C8" s="5" t="n">
         <v>850.66</v>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" t="inlineStr">
+    <row r="9">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Vienna — Hotel Marc Aurel, 2 nights (Jul 19–21)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C9" s="5" t="n">
         <v>609</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C10" s="8">
+        <f>SUM(C6:C9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Airport → city: MVV group day ticket *</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C12" s="5" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="5" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Bayern-Ticket: Munich → Berchtesgaden (Jul 14, group) *</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C13" s="5" t="n">
         <v>33</v>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="5" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>ÖBB Railjet: Salzburg → Vienna (Jul 18, 4 people) *</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C14" s="5" t="n">
         <v>110</v>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Vienna public transit *</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C15" s="5" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C16" s="8">
+        <f>SUM(C12:C15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Activities</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Mike's Bike Tours Munich (4 people) *</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C18" s="5" t="n">
         <v>160</v>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="5" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Nymphenburg Palace admission (4 people) *</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C19" s="5" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="5" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Eagle's Nest Kehlstein bus (4 people) *</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C20" s="5" t="n">
         <v>80</v>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Königssee electric boat (4 people) *</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C21" s="5" t="n">
         <v>88</v>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="5" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Hohensalzburg fortress admission (4 people) *</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C22" s="5" t="n">
         <v>66</v>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="5" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>St. Peter Stiftskeller dinner (4 people) *</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C23" s="5" t="n">
         <v>220</v>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="5" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Schönbrunn Palace + maze (4 people) *</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C24" s="5" t="n">
         <v>132</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C25" s="8">
+        <f>SUM(C18:C24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Meals &amp; Incidentals</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Meals (~$150/day × 10 days) *</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C27" s="5" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="5" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Miscellaneous / buffer *</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C28" s="5" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C29" s="8">
+        <f>SUM(C27:C28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="8">
-        <f>SUM(C2:C24)</f>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="12">
+        <f>C4+C10+C16+C25+C29</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>* = estimated</t>
         </is>

</xml_diff>

<commit_message>
Fix transport costs: add missing legs and correct Bayern-Ticket amount
Added: local buses Berchtesgaden (Days 4-5), Schönau→Salzburg Leg 3
(Jul 17), CAT airport train Vienna (Jul 21). Fixed Bayern-Ticket from
$33 to $58 (~EUR 53 as shown in itinerary). Transport: $181 -> $386.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trip_costs.xlsx
+++ b/trip_costs.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -593,7 +593,7 @@
     <row r="12">
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Airport → city: MVV group day ticket *</t>
+          <t>Airport → city: MVV group day ticket (Jul 12) *</t>
         </is>
       </c>
       <c r="C12" s="5" t="n">
@@ -607,187 +607,217 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>33</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>ÖBB Railjet: Salzburg → Vienna (Jul 18, 4 people) *</t>
+          <t>Local buses Berchtesgaden area (Jul 15–16, ~€8/day) *</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>110</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Vienna public transit *</t>
+          <t>Schönau → Salzburg: taxi to Freilassing + ÖBB (Jul 17) *</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>ÖBB Railjet: Salzburg → Vienna (Jul 19, 4 people) *</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Vienna public transit (Jul 19–21) *</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
         <v>22</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="C16" s="8">
-        <f>SUM(C12:C15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Activities</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Mike's Bike Tours Munich (4 people) *</t>
+          <t>CAT Wien Mitte → VIE airport (Jul 21, 4 people) *</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>160</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Nymphenburg Palace admission (4 people) *</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>44</v>
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C19" s="8">
+        <f>SUM(C12:C18)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Eagle's Nest Kehlstein bus (4 people) *</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>80</v>
-      </c>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Activities</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Königssee electric boat (4 people) *</t>
+          <t>Mike's Bike Tours Munich (4 people) *</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>88</v>
+        <v>160</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Hohensalzburg fortress admission (4 people) *</t>
+          <t>Nymphenburg Palace admission (4 people) *</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>St. Peter Stiftskeller dinner (4 people) *</t>
+          <t>Eagle's Nest Kehlstein bus (4 people) *</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>220</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Schönbrunn Palace + maze (4 people) *</t>
+          <t>Königssee electric boat (4 people) *</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>132</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="C25" s="8">
-        <f>SUM(C18:C24)</f>
-        <v/>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Hohensalzburg fortress admission (4 people) *</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>66</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Meals &amp; Incidentals</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>St. Peter Stiftskeller dinner (4 people) *</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="9" t="inlineStr">
         <is>
+          <t>Schönbrunn Palace + maze (4 people) *</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C28" s="8">
+        <f>SUM(C21:C27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Meals &amp; Incidentals</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="9" t="inlineStr">
+        <is>
           <t>Meals (~$150/day × 10 days) *</t>
         </is>
       </c>
-      <c r="C27" s="5" t="n">
+      <c r="C30" s="5" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="9" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>Miscellaneous / buffer *</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n">
+      <c r="C31" s="5" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="7" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="6" t="n"/>
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="C29" s="8">
-        <f>SUM(C27:C28)</f>
+      <c r="C32" s="8">
+        <f>SUM(C30:C31)</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="12">
-        <f>C4+C10+C16+C25+C29</f>
+      <c r="B34" s="11" t="n"/>
+      <c r="C34" s="12">
+        <f>C4+C10+C19+C28+C32</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>* = estimated</t>
         </is>

</xml_diff>

<commit_message>
Move category subtotals to header row in cost table
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trip_costs.xlsx
+++ b/trip_costs.xlsx
@@ -45,7 +45,7 @@
       <color rgb="00888888"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -62,11 +62,6 @@
         <fgColor rgb="00D5E8F5"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EAF3FB"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -80,18 +75,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -464,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -496,328 +489,283 @@
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-    </row>
-    <row r="3">
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>UA 108 IAD→MUC Jul 11 + OS135/UA53 VIE→IAD Jul 21 (4 people, Standard Economy)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>5422.52</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="C4" s="8">
+      <c r="C2" s="4">
         <f>SUM(C3:C3)</f>
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>UA 108 IAD→MUC Jul 11 + OS135/UA53 VIE→IAD Jul 21 (4 people, Standard Economy)</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>5422.52</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="4">
+        <f>SUM(C5:C8)</f>
+        <v/>
+      </c>
+    </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Accommodation</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Munich — Holiday Inn Westpark, 2 nights (Jul 12–14)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>677.36</v>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Munich — Holiday Inn Westpark, 2 nights (Jul 12–14)</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>677.36</v>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Königssee — Villa Alpenrausch, 3 nights (Jul 14–17) *</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Königssee — Villa Alpenrausch, 3 nights (Jul 14–17) *</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Salzburg — Numa Vogelweider, 2 nights (Jul 17–19)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>850.66</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Vienna — Hotel Marc Aurel, 2 nights (Jul 19–21)</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="4">
+        <f>SUM(C10:C16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Airport → city: MVV group day ticket (Jul 12) *</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Bayern-Ticket: Munich → Berchtesgaden (Jul 14, group) *</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Local buses Berchtesgaden area (Jul 15–16, ~€8/day) *</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Schönau → Salzburg: taxi to Freilassing + ÖBB (Jul 17) *</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>ÖBB Railjet: Salzburg → Vienna (Jul 19, 4 people) *</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Vienna public transit (Jul 19–21) *</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>CAT Wien Mitte → VIE airport (Jul 21, 4 people) *</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Activities</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="4">
+        <f>SUM(C18:C24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Mike's Bike Tours Munich (4 people) *</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Nymphenburg Palace admission (4 people) *</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Eagle's Nest Kehlstein bus (4 people) *</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Königssee electric boat (4 people) *</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Hohensalzburg fortress admission (4 people) *</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>St. Peter Stiftskeller dinner (4 people) *</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Schönbrunn Palace + maze (4 people) *</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Meals &amp; Incidentals</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="4">
+        <f>SUM(C26:C27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Meals (~$150/day × 10 days) *</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Salzburg — Numa Vogelweider, 2 nights (Jul 17–19)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>850.66</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Vienna — Hotel Marc Aurel, 2 nights (Jul 19–21)</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>609</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="C10" s="8">
-        <f>SUM(C6:C9)</f>
+    <row r="27">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Miscellaneous / buffer *</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="n"/>
+      <c r="C29" s="10">
+        <f>C2+C4+C9+C17+C25</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Airport → city: MVV group day ticket (Jul 12) *</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Bayern-Ticket: Munich → Berchtesgaden (Jul 14, group) *</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Local buses Berchtesgaden area (Jul 15–16, ~€8/day) *</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Schönau → Salzburg: taxi to Freilassing + ÖBB (Jul 17) *</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>ÖBB Railjet: Salzburg → Vienna (Jul 19, 4 people) *</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Vienna public transit (Jul 19–21) *</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>CAT Wien Mitte → VIE airport (Jul 21, 4 people) *</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="C19" s="8">
-        <f>SUM(C12:C18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Activities</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Mike's Bike Tours Munich (4 people) *</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Nymphenburg Palace admission (4 people) *</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Eagle's Nest Kehlstein bus (4 people) *</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Königssee electric boat (4 people) *</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Hohensalzburg fortress admission (4 people) *</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>St. Peter Stiftskeller dinner (4 people) *</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Schönbrunn Palace + maze (4 people) *</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="C28" s="8">
-        <f>SUM(C21:C27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Meals &amp; Incidentals</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Meals (~$150/day × 10 days) *</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>1500</v>
-      </c>
-    </row>
     <row r="31">
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>Miscellaneous / buffer *</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="C32" s="8">
-        <f>SUM(C30:C31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="n"/>
-      <c r="C34" s="12">
-        <f>C4+C10+C19+C28+C32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>* = estimated</t>
         </is>

</xml_diff>

<commit_message>
Add bookings.md; update itinerary for Jul 11-22, confirmed flights/accommodations/activities
- New bookings.md: confirmed flights (IKR3ZV), Villa Alpenrausch, Mike's Bike Tours, Nymphenburg Palace
- Trip extended to Jul 11-22 (Vienna 3 nights); all dates updated throughout
- Day 3 Nymphenburg restructured for 9 AM entry + Palmenhaus lunch; 14:44 train
- Flights updated: OS 41 nonstop VIE→IAD Jul 22
- Accommodation: Villa Alpenrausch confirmed $1,435.99; dropped Schiffmeister/Alpenveilchen options
- build_costs.py: mark flights, Villa Alpenrausch, Mike's Bikes, Nymphenburg as confirmed
- CLAUDE.md: updated dates, added bookings.md entry, split scripts section

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trip_costs.xlsx
+++ b/trip_costs.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>UA 108 IAD→MUC Jul 11 + OS135/UA53 VIE→IAD Jul 21 (4 people, Standard Economy)</t>
+          <t>UA 108 IAD→MUC Jul 11 + OS 41 VIE→IAD Jul 22 nonstop (4 people) — Conf. IKR3ZV</t>
         </is>
       </c>
       <c r="C3" s="6" t="n">
@@ -527,13 +527,13 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Königssee — Villa Alpenrausch, 3 nights (Jul 14–17) *</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Königssee — Villa Alpenrausch, 3 nights (Jul 14–17) BOOKED</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>1500</v>
+        <v>1435.99</v>
       </c>
     </row>
     <row r="7">
@@ -547,13 +547,13 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Vienna — Hotel Marc Aurel, 2 nights (Jul 19–21)</t>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Vienna — hotel TBD, 3 nights (Jul 19–22) *</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>609</v>
+        <v>900</v>
       </c>
     </row>
     <row r="9">
@@ -621,17 +621,17 @@
     <row r="15">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Vienna public transit (Jul 19–21) *</t>
+          <t>Vienna public transit (Jul 19–22) *</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>CAT Wien Mitte → VIE airport (Jul 21, 4 people) *</t>
+          <t>CAT Wien Mitte → VIE airport (Jul 22, 4 people) *</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
@@ -646,28 +646,28 @@
       </c>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="4">
-        <f>SUM(C18:C24)</f>
+        <f>SUM(C18:C26)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Mike's Bike Tours Munich (4 people) *</t>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Mike's Bike Tours Munich (4 people) — €180.67 paid, Booking #354406124</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>160</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Nymphenburg Palace admission (4 people) *</t>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Nymphenburg Palace combination ticket — €58 paid, Order #42616</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>44</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20">
@@ -721,51 +721,71 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Meals &amp; Incidentals</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="4">
-        <f>SUM(C26:C27)</f>
-        <v/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Upper Belvedere admission (4 people) *</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>84</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Meals (~$150/day × 10 days) *</t>
+          <t>Riesenrad / Prater (4 people) *</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>1500</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="7" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Meals &amp; Incidentals</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="4">
+        <f>SUM(C28:C29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Meals (~$150/day × 11 days) *</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Miscellaneous / buffer *</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C29" s="6" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B29" s="9" t="n"/>
-      <c r="C29" s="10">
-        <f>C2+C4+C9+C17+C25</f>
+      <c r="B31" s="9" t="n"/>
+      <c r="C31" s="10">
+        <f>C2+C4+C9+C17+C27</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>* = estimated</t>
         </is>

</xml_diff>

<commit_message>
Add Vienna Airbnb + Salzburg Airbnb bookings; confirm all accommodation
- Vienna: City Center Klimt's Balcony Suite (Conf. HMT8SQRKMA, $1,068.21, Jul 19-22)
- Salzburg: Mozart House Gstättengasse 25 (Conf. HM4NSFM9J3, $1,007.28, Jul 17-19)
- All four accommodations now confirmed; trip total $13,252
- Corrected Day 8 train timing (10:07 AM is fine; checkout by 10 AM means leave early)
- Added itinerary_share.html (no-pricing shareable version)
- Updated CLAUDE.md, build_costs.py, bookings.md, itinerary.md, itinerary.html

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trip_costs.xlsx
+++ b/trip_costs.xlsx
@@ -519,11 +519,11 @@
     <row r="5">
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Munich — Holiday Inn Westpark, 2 nights (Jul 12–14)</t>
+          <t>Munich — PRIME City Apt Adamstraße 4, 2 nights (Jul 12–14) — Conf. HM4ZPJHYB9</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>677.36</v>
+        <v>782.08</v>
       </c>
     </row>
     <row r="6">
@@ -539,21 +539,21 @@
     <row r="7">
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Salzburg — Numa Vogelweider, 2 nights (Jul 17–19)</t>
+          <t>Salzburg — Mozart House Gstättengasse 25, 2 nights (Jul 17–19) — Conf. HM4NSFM9J3</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>850.66</v>
+        <v>1007.28</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Vienna — hotel TBD, 3 nights (Jul 19–22) *</t>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Vienna — City Center Klimt's Balcony Suite, 3 nights (Jul 19–22) — Conf. HMT8SQRKMA</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>900</v>
+        <v>1068.21</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Sync confirmed bookings and trip costs
</commit_message>
<xml_diff>
--- a/trip_costs.xlsx
+++ b/trip_costs.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -564,7 +564,7 @@
       </c>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="4">
-        <f>SUM(C10:C16)</f>
+        <f>SUM(C10:C18)</f>
         <v/>
       </c>
     </row>
@@ -579,213 +579,233 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Bayern-Ticket: Munich → Berchtesgaden (Jul 14, group) *</t>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Bayern-Ticket: Munich → Berchtesgaden (Jul 14, group) — €64.00 paid, Conf. 342448586457</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>58</v>
+        <v>69.76000000000001</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Local buses Berchtesgaden area (Jul 15–16, ~€8/day) *</t>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Bounce luggage storage, Munich (Jul 12, 4 reg + 4 small bags) — €40.80 paid, Ref S69FQ16J</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>18</v>
+        <v>44.47</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Schönau → Salzburg: taxi to Freilassing + ÖBB (Jul 17) *</t>
+          <t>Local buses Berchtesgaden area (Jul 15–16, ~€8/day) *</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>100</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>ÖBB Railjet: Salzburg → Vienna (Jul 19, 4 people) *</t>
+          <t>Schönau → Salzburg: taxi to Freilassing + ÖBB (Jul 17) *</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>WESTbahn: Salzburg → Vienna (Jul 19, 4 people) — Conf. NAYRKY</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>262.84</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Bounce luggage storage, Vienna (Jul 19, 4 reg + 4 small bags) — €30.27 paid, Ref 1X9XMXPG</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>32.99</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Vienna public transit (Jul 19–22) *</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C17" s="6" t="n">
         <v>28</v>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="7" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>CAT Wien Mitte → VIE airport (Jul 22, 4 people) *</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C18" s="6" t="n">
         <v>52</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Activities</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="4">
-        <f>SUM(C18:C26)</f>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="4">
+        <f>SUM(C20:C28)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Mike's Bike Tours Munich (4 people) — €180.67 paid, Booking #354406124</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C20" s="6" t="n">
         <v>197</v>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="5" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Nymphenburg Palace combination ticket — €58 paid, Order #42616</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C21" s="6" t="n">
         <v>63</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Eagle's Nest Kehlstein bus (4 people) *</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Königssee electric boat (4 people) *</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>88</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Hohensalzburg fortress admission (4 people) *</t>
+          <t>Eagle's Nest Kehlstein bus (4 people) *</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>66</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>St. Peter Stiftskeller dinner (4 people) *</t>
+          <t>Königssee electric boat (4 people) *</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>220</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Schönbrunn Palace + maze (4 people) *</t>
+          <t>Hohensalzburg fortress admission (4 people) *</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Upper Belvedere admission (4 people) *</t>
+          <t>St. Peter Stiftskeller dinner (4 people) *</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>84</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Riesenrad / Prater (4 people) *</t>
+          <t>Schönbrunn Palace + maze (4 people) *</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>64</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Meals &amp; Incidentals</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="4">
-        <f>SUM(C28:C29)</f>
-        <v/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Upper Belvedere admission (4 people) *</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>84</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="7" t="inlineStr">
         <is>
+          <t>Riesenrad / Prater (4 people) *</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Meals &amp; Incidentals</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="4">
+        <f>SUM(C30:C31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
           <t>Meals (~$150/day × 11 days) *</t>
         </is>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C30" s="6" t="n">
         <v>1650</v>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="7" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Miscellaneous / buffer *</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C31" s="6" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="10">
-        <f>C2+C4+C9+C17+C27</f>
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="10">
+        <f>C2+C4+C9+C19+C29</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>* = estimated</t>
         </is>

</xml_diff>

<commit_message>
Add Salzburg storage and Eagle Nest transit plan
</commit_message>
<xml_diff>
--- a/trip_costs.xlsx
+++ b/trip_costs.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -564,7 +564,7 @@
       </c>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="4">
-        <f>SUM(C10:C18)</f>
+        <f>SUM(C10:C19)</f>
         <v/>
       </c>
     </row>
@@ -599,19 +599,19 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Local buses Berchtesgaden area (Jul 15–16, ~€8/day) *</t>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Berchtesgaden local RVO buses — included with host-provided Guest Card (line 849 excluded)</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Schönau → Salzburg: taxi to Freilassing + ÖBB (Jul 17) *</t>
+          <t>Schönau → Salzburg: direct taxi (Jul 17) *</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
@@ -621,191 +621,201 @@
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>WESTbahn: Salzburg → Vienna (Jul 19, 4 people) — Conf. NAYRKY</t>
+          <t>Bounce luggage storage, Salzburg (Jul 17, 4 reg + 4 small bags) — €48.80 paid, Ref 543WH67Q</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>262.84</v>
+        <v>53.19</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
+          <t>WESTbahn: Salzburg → Vienna (Jul 19, 4 people) — Conf. NAYRKY</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>262.84</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
           <t>Bounce luggage storage, Vienna (Jul 19, 4 reg + 4 small bags) — €30.27 paid, Ref 1X9XMXPG</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C17" s="6" t="n">
         <v>32.99</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Vienna public transit (Jul 19–22) *</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>28</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
+          <t>Vienna public transit (Jul 19–22) *</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
           <t>CAT Wien Mitte → VIE airport (Jul 22, 4 people) *</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C19" s="6" t="n">
         <v>52</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Activities</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="4">
-        <f>SUM(C20:C28)</f>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="4">
+        <f>SUM(C21:C29)</f>
         <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Mike's Bike Tours Munich (4 people) — €180.67 paid, Booking #354406124</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>197</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
+          <t>Mike's Bike Tours Munich (4 people) — €180.67 paid, Booking #354406124</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
           <t>Nymphenburg Palace combination ticket — €58 paid, Order #42616</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C22" s="6" t="n">
         <v>63</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Eagle's Nest Kehlstein bus (4 people) *</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>80</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Königssee electric boat (4 people) *</t>
+          <t>Eagle's Nest Kehlstein bus (4 people) *</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Hohensalzburg fortress admission (4 people) *</t>
+          <t>Königssee electric boat (4 people) *</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>66</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>St. Peter Stiftskeller dinner (4 people) *</t>
+          <t>Hohensalzburg fortress admission (4 people) *</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>220</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Schönbrunn Palace + maze (4 people) *</t>
+          <t>St. Peter Stiftskeller dinner (4 people) *</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>132</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Upper Belvedere admission (4 people) *</t>
+          <t>Schönbrunn Palace + maze (4 people) *</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>84</v>
+        <v>132</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="7" t="inlineStr">
         <is>
+          <t>Upper Belvedere admission (4 people) *</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="7" t="inlineStr">
+        <is>
           <t>Riesenrad / Prater (4 people) *</t>
         </is>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C29" s="6" t="n">
         <v>64</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Meals &amp; Incidentals</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="4">
-        <f>SUM(C30:C31)</f>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="4">
+        <f>SUM(C31:C32)</f>
         <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Meals (~$150/day × 11 days) *</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n">
-        <v>1650</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="7" t="inlineStr">
         <is>
+          <t>Meals (~$150/day × 11 days) *</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
           <t>Miscellaneous / buffer *</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C32" s="6" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="10">
-        <f>C2+C4+C9+C19+C29</f>
+      <c r="B34" s="9" t="n"/>
+      <c r="C34" s="10">
+        <f>C2+C4+C9+C20+C30</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>* = estimated</t>
         </is>

</xml_diff>

<commit_message>
add Taxi Angerer details
</commit_message>
<xml_diff>
--- a/trip_costs.xlsx
+++ b/trip_costs.xlsx
@@ -609,13 +609,13 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Schönau → Salzburg: direct taxi (Jul 17) *</t>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Schönau → Salzburg: Taxi Angerer (Jul 17) — €75.00 paid</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>100</v>
+        <v>81.75</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Rework Berchtesgaden hiking days
</commit_message>
<xml_diff>
--- a/trip_costs.xlsx
+++ b/trip_costs.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -564,7 +564,7 @@
       </c>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="4">
-        <f>SUM(C10:C19)</f>
+        <f>SUM(C10:C20)</f>
         <v/>
       </c>
     </row>
@@ -609,213 +609,233 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Schönau → Salzburg: Taxi Angerer (Jul 17) — €75.00 paid</t>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Day 4 taxis: Zechmeister → Wimbachbrücke → Berchtesgaden salt mine *</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>81.75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Bounce luggage storage, Salzburg (Jul 17, 4 reg + 4 small bags) — €48.80 paid, Ref 543WH67Q</t>
+          <t>Schönau → Salzburg: Taxi Angerer (Jul 17) — €75.00 paid</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>53.19</v>
+        <v>81.75</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>WESTbahn: Salzburg → Vienna (Jul 19, 4 people) — Conf. NAYRKY</t>
+          <t>Bounce luggage storage, Salzburg (Jul 17, 4 reg + 4 small bags) — €48.80 paid, Ref 543WH67Q</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>262.84</v>
+        <v>53.19</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
         <is>
+          <t>WESTbahn: Salzburg → Vienna (Jul 19, 4 people) — Conf. NAYRKY</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>262.84</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
           <t>Bounce luggage storage, Vienna (Jul 19, 4 reg + 4 small bags) — €30.27 paid, Ref 1X9XMXPG</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C18" s="6" t="n">
         <v>32.99</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Vienna public transit (Jul 19–22) *</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>28</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
+          <t>Vienna public transit (Jul 19–22) *</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
           <t>CAT Wien Mitte → VIE airport (Jul 22, 4 people) *</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C20" s="6" t="n">
         <v>52</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Activities</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="4">
-        <f>SUM(C21:C29)</f>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="4">
+        <f>SUM(C22:C31)</f>
         <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Mike's Bike Tours Munich (4 people) — €180.67 paid, Booking #354406124</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>197</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
         <is>
+          <t>Mike's Bike Tours Munich (4 people) — €180.67 paid, Booking #354406124</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
           <t>Nymphenburg Palace combination ticket — €58 paid, Order #42616</t>
         </is>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C23" s="6" t="n">
         <v>63</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Eagle's Nest Kehlstein bus (4 people) *</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>80</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Königssee electric boat (4 people) *</t>
+          <t>Optional Eagle's Nest game-time audible: Kehlstein bus (4 people) *</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Hohensalzburg fortress admission (4 people) *</t>
+          <t>Wimbachklamm gorge admission (4 people) *</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>66</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>St. Peter Stiftskeller dinner (4 people) *</t>
+          <t>Königssee electric boat (4 people) *</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>220</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Schönbrunn Palace + maze (4 people) *</t>
+          <t>Hohensalzburg fortress admission (4 people) *</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Upper Belvedere admission (4 people) *</t>
+          <t>St. Peter Stiftskeller dinner (4 people) *</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>84</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Riesenrad / Prater (4 people) *</t>
+          <t>Schönbrunn Palace + maze (4 people) *</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>64</v>
+        <v>132</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Meals &amp; Incidentals</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="4">
-        <f>SUM(C31:C32)</f>
-        <v/>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Upper Belvedere admission (4 people) *</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>84</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="7" t="inlineStr">
         <is>
+          <t>Riesenrad / Prater (4 people) *</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Meals &amp; Incidentals</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="4">
+        <f>SUM(C33:C34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
           <t>Meals (~$150/day × 11 days) *</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C33" s="6" t="n">
         <v>1650</v>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="7" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>Miscellaneous / buffer *</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n">
+      <c r="C34" s="6" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B34" s="9" t="n"/>
-      <c r="C34" s="10">
-        <f>C2+C4+C9+C20+C30</f>
+      <c r="B36" s="9" t="n"/>
+      <c r="C36" s="10">
+        <f>C2+C4+C9+C21+C32</f>
         <v/>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>* = estimated</t>
         </is>

</xml_diff>